<commit_message>
New changes done - Feb 24, 26
</commit_message>
<xml_diff>
--- a/SalamtekAutomation_v1/TestData/TestData_DEV.xlsx
+++ b/SalamtekAutomation_v1/TestData/TestData_DEV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\g.barried\git\Salamtek_Web_v1\SalamtekAutomation_v1\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A1BDD7E-83CC-4B6B-A3A1-835938DA5E51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F68E64B0-CBB5-49AA-B367-056B342F1791}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="6" xr2:uid="{BA93E413-0FBB-4423-B223-0A6D5A2FA904}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5411" uniqueCount="1042">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5451" uniqueCount="1048">
   <si>
     <t>TestCaseName</t>
   </si>
@@ -3187,6 +3187,24 @@
   </si>
   <si>
     <t>COMPLETE YOUR ORDER NOW</t>
+  </si>
+  <si>
+    <t>SLMTK_T1349</t>
+  </si>
+  <si>
+    <t>Admin_Promo_Cancel_Pharmacy</t>
+  </si>
+  <si>
+    <t>Verify whether user is able to get the correct refund while cancelling discounted product with promo</t>
+  </si>
+  <si>
+    <t>FAY SERUM</t>
+  </si>
+  <si>
+    <t>proForPharmacy_853</t>
+  </si>
+  <si>
+    <t>#100006256</t>
   </si>
 </sst>
 </file>
@@ -14638,7 +14656,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A3A20B8-DAEA-4FEF-8D62-6F90EBCAE657}">
-  <dimension ref="A1:BR22"/>
+  <dimension ref="A1:BR23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1" collapsed="1"/>
@@ -17502,6 +17520,143 @@
         <v>737</v>
       </c>
     </row>
+    <row r="23" spans="1:70" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>1042</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>1043</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>1044</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>687</v>
+      </c>
+      <c r="P23" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q23" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="R23" s="3" t="s">
+        <v>751</v>
+      </c>
+      <c r="U23" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="V23" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="W23" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="X23" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="Y23" s="12" t="s">
+        <v>607</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>608</v>
+      </c>
+      <c r="AB23" t="s">
+        <v>637</v>
+      </c>
+      <c r="AC23" s="5" t="s">
+        <v>711</v>
+      </c>
+      <c r="AD23" t="s">
+        <v>637</v>
+      </c>
+      <c r="AE23" t="s">
+        <v>613</v>
+      </c>
+      <c r="AF23" s="5" t="s">
+        <v>615</v>
+      </c>
+      <c r="AG23" s="5" t="s">
+        <v>627</v>
+      </c>
+      <c r="AH23" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="AI23" s="5" t="s">
+        <v>421</v>
+      </c>
+      <c r="AR23" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="AS23" s="3" t="s">
+        <v>1045</v>
+      </c>
+      <c r="AU23" t="s">
+        <v>45</v>
+      </c>
+      <c r="AV23" t="s">
+        <v>45</v>
+      </c>
+      <c r="BE23">
+        <v>55</v>
+      </c>
+      <c r="BF23">
+        <v>52.5</v>
+      </c>
+      <c r="BG23">
+        <v>2.5</v>
+      </c>
+      <c r="BH23" t="s">
+        <v>1046</v>
+      </c>
+      <c r="BI23" t="s">
+        <v>737</v>
+      </c>
+      <c r="BJ23">
+        <v>2450.3470000000002</v>
+      </c>
+      <c r="BK23">
+        <v>2502.6469999999999</v>
+      </c>
+      <c r="BL23" t="s">
+        <v>737</v>
+      </c>
+      <c r="BM23" t="s">
+        <v>737</v>
+      </c>
+      <c r="BN23" t="s">
+        <v>737</v>
+      </c>
+      <c r="BO23" t="s">
+        <v>737</v>
+      </c>
+      <c r="BP23" t="s">
+        <v>1047</v>
+      </c>
+      <c r="BQ23" t="s">
+        <v>26</v>
+      </c>
+      <c r="BR23" t="s">
+        <v>737</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:BR21" xr:uid="{5A3A20B8-DAEA-4FEF-8D62-6F90EBCAE657}"/>
   <hyperlinks>
@@ -17526,6 +17681,7 @@
     <hyperlink ref="W20" r:id="rId19" xr:uid="{AC229CC6-F7F5-4BE3-9BCA-628BFFC2F6D8}"/>
     <hyperlink ref="W21" r:id="rId20" xr:uid="{AC8D1D43-C0D3-42D6-BE8B-19C32507E0A4}"/>
     <hyperlink ref="W22" r:id="rId21" xr:uid="{E3F8960F-4B96-42DF-B7B9-A18E25179D43}"/>
+    <hyperlink ref="W23" r:id="rId22" xr:uid="{344412D7-6104-4963-8F0B-242ED8731857}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>